<commit_message>
Switch product mapping to 판매중_상품구성_사업방법서_매핑.xlsx
- batch_run.py: 기존 키워드 추론 방식 제거, 파일명 직접 조회로 교체
  - load_mapping_db(): 새 매핑 파일 로드
  - get_pdf_entries(): 파일명으로 DTCD+ITCD 직접 반환
  - 복수 DTCD PDF 지원 (1 PDF → N DTCD 처리)
- CLAUDE.md: STEP 2 설명을 직접 매핑 조회 방식으로 업데이트
- 검증 결과: PASS 11개 유지

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/upload/S00022_1228_연금저축_스마트하이드림연금보험.xlsx
+++ b/output/upload/S00022_1228_연금저축_스마트하이드림연금보험.xlsx
@@ -1372,17 +1372,9 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n"/>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>1228133</t>
-        </is>
-      </c>
+      <c r="B7" s="5" t="inlineStr"/>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>1228133</t>
-        </is>
-      </c>
+      <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Improve S00022/S00027 extraction accuracy (session 7-8)
- extraction_rules.py: add N-type year pattern for 보기개시나이 (종신보험류 N2/N3/N5/N6/N8/N10)
- extraction_rules.py: add pattern 0 for multi-종 연금개시나이 table (1종: X55~X80, 2종: X55~X110)
- extraction_rules.py: expand 전기납 → X{연금개시나이} PP codes for S00027
- convert_codes.py: support N-type in convert_s00022 (SPIN_STRT_DVSN_CODE='N')
- generate_report.py: filter GT by mapped ITCDs for S00022 comparison

Results: S00022 일치 19/불일치 0, S00027 일치 48, S00028 일치 56 (100%)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/upload/S00022_1228_연금저축_스마트하이드림연금보험.xlsx
+++ b/output/upload/S00022_1228_연금저축_스마트하이드림연금보험.xlsx
@@ -1416,13 +1416,21 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
+      <c r="B8" s="5" t="inlineStr"/>
       <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
+      <c r="D8" s="5" t="inlineStr"/>
       <c r="E8" s="5" t="n"/>
       <c r="F8" s="5" t="n"/>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
@@ -1432,7 +1440,11 @@
       <c r="O8" s="6" t="n"/>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="6" t="n"/>
+      <c r="R8" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S8" s="6" t="n"/>
       <c r="T8" s="6" t="n"/>
       <c r="U8" s="6" t="n"/>
@@ -1448,13 +1460,21 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="n"/>
+      <c r="B9" s="5" t="inlineStr"/>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
+      <c r="D9" s="5" t="inlineStr"/>
       <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
@@ -1464,7 +1484,11 @@
       <c r="O9" s="6" t="n"/>
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="6" t="n"/>
-      <c r="R9" s="6" t="n"/>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S9" s="6" t="n"/>
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="n"/>
@@ -1480,13 +1504,21 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
+      <c r="B10" s="5" t="inlineStr"/>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
+      <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I10" s="6" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
@@ -1496,7 +1528,11 @@
       <c r="O10" s="6" t="n"/>
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="6" t="n"/>
+      <c r="R10" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S10" s="6" t="n"/>
       <c r="T10" s="6" t="n"/>
       <c r="U10" s="6" t="n"/>
@@ -1512,13 +1548,21 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="n"/>
+      <c r="B11" s="5" t="inlineStr"/>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
+      <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
-      <c r="G11" s="6" t="n"/>
-      <c r="H11" s="6" t="n"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
@@ -1528,7 +1572,11 @@
       <c r="O11" s="6" t="n"/>
       <c r="P11" s="6" t="n"/>
       <c r="Q11" s="6" t="n"/>
-      <c r="R11" s="6" t="n"/>
+      <c r="R11" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S11" s="6" t="n"/>
       <c r="T11" s="6" t="n"/>
       <c r="U11" s="6" t="n"/>
@@ -1544,13 +1592,21 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
+      <c r="B12" s="5" t="inlineStr"/>
       <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
+      <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="n"/>
-      <c r="G12" s="6" t="n"/>
-      <c r="H12" s="6" t="n"/>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
@@ -1560,7 +1616,11 @@
       <c r="O12" s="6" t="n"/>
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="6" t="n"/>
+      <c r="R12" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S12" s="6" t="n"/>
       <c r="T12" s="6" t="n"/>
       <c r="U12" s="6" t="n"/>
@@ -1576,13 +1636,21 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="n"/>
+      <c r="B13" s="5" t="inlineStr"/>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
+      <c r="D13" s="5" t="inlineStr"/>
       <c r="E13" s="5" t="n"/>
       <c r="F13" s="5" t="n"/>
-      <c r="G13" s="6" t="n"/>
-      <c r="H13" s="6" t="n"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
@@ -1592,7 +1660,11 @@
       <c r="O13" s="6" t="n"/>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="6" t="n"/>
+      <c r="R13" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S13" s="6" t="n"/>
       <c r="T13" s="6" t="n"/>
       <c r="U13" s="6" t="n"/>
@@ -1608,13 +1680,21 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="n"/>
+      <c r="B14" s="5" t="inlineStr"/>
       <c r="C14" s="5" t="n"/>
-      <c r="D14" s="5" t="n"/>
+      <c r="D14" s="5" t="inlineStr"/>
       <c r="E14" s="5" t="n"/>
       <c r="F14" s="5" t="n"/>
-      <c r="G14" s="6" t="n"/>
-      <c r="H14" s="6" t="n"/>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
@@ -1624,7 +1704,11 @@
       <c r="O14" s="6" t="n"/>
       <c r="P14" s="6" t="n"/>
       <c r="Q14" s="6" t="n"/>
-      <c r="R14" s="6" t="n"/>
+      <c r="R14" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S14" s="6" t="n"/>
       <c r="T14" s="6" t="n"/>
       <c r="U14" s="6" t="n"/>
@@ -1640,13 +1724,21 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="n"/>
+      <c r="B15" s="5" t="inlineStr"/>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
+      <c r="D15" s="5" t="inlineStr"/>
       <c r="E15" s="5" t="n"/>
       <c r="F15" s="5" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
@@ -1656,7 +1748,11 @@
       <c r="O15" s="6" t="n"/>
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="6" t="n"/>
-      <c r="R15" s="6" t="n"/>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S15" s="6" t="n"/>
       <c r="T15" s="6" t="n"/>
       <c r="U15" s="6" t="n"/>
@@ -1672,13 +1768,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="n"/>
+      <c r="B16" s="5" t="inlineStr"/>
       <c r="C16" s="5" t="n"/>
-      <c r="D16" s="5" t="n"/>
+      <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="5" t="n"/>
       <c r="F16" s="5" t="n"/>
-      <c r="G16" s="6" t="n"/>
-      <c r="H16" s="6" t="n"/>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I16" s="6" t="n"/>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
@@ -1688,7 +1792,11 @@
       <c r="O16" s="6" t="n"/>
       <c r="P16" s="6" t="n"/>
       <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="6" t="n"/>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S16" s="6" t="n"/>
       <c r="T16" s="6" t="n"/>
       <c r="U16" s="6" t="n"/>
@@ -1704,13 +1812,21 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="n"/>
+      <c r="B17" s="5" t="inlineStr"/>
       <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
+      <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="5" t="n"/>
       <c r="F17" s="5" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
@@ -1720,7 +1836,11 @@
       <c r="O17" s="6" t="n"/>
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="6" t="n"/>
-      <c r="R17" s="6" t="n"/>
+      <c r="R17" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S17" s="6" t="n"/>
       <c r="T17" s="6" t="n"/>
       <c r="U17" s="6" t="n"/>
@@ -1736,13 +1856,21 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="n"/>
+      <c r="B18" s="5" t="inlineStr"/>
       <c r="C18" s="5" t="n"/>
-      <c r="D18" s="5" t="n"/>
+      <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="5" t="n"/>
       <c r="F18" s="5" t="n"/>
-      <c r="G18" s="6" t="n"/>
-      <c r="H18" s="6" t="n"/>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
@@ -1752,7 +1880,11 @@
       <c r="O18" s="6" t="n"/>
       <c r="P18" s="6" t="n"/>
       <c r="Q18" s="6" t="n"/>
-      <c r="R18" s="6" t="n"/>
+      <c r="R18" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S18" s="6" t="n"/>
       <c r="T18" s="6" t="n"/>
       <c r="U18" s="6" t="n"/>
@@ -1768,13 +1900,21 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="n"/>
+      <c r="B19" s="5" t="inlineStr"/>
       <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
+      <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="5" t="n"/>
       <c r="F19" s="5" t="n"/>
-      <c r="G19" s="6" t="n"/>
-      <c r="H19" s="6" t="n"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
@@ -1784,7 +1924,11 @@
       <c r="O19" s="6" t="n"/>
       <c r="P19" s="6" t="n"/>
       <c r="Q19" s="6" t="n"/>
-      <c r="R19" s="6" t="n"/>
+      <c r="R19" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S19" s="6" t="n"/>
       <c r="T19" s="6" t="n"/>
       <c r="U19" s="6" t="n"/>
@@ -1800,13 +1944,21 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="n"/>
+      <c r="B20" s="5" t="inlineStr"/>
       <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
+      <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="5" t="n"/>
       <c r="F20" s="5" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
@@ -1816,7 +1968,11 @@
       <c r="O20" s="6" t="n"/>
       <c r="P20" s="6" t="n"/>
       <c r="Q20" s="6" t="n"/>
-      <c r="R20" s="6" t="n"/>
+      <c r="R20" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S20" s="6" t="n"/>
       <c r="T20" s="6" t="n"/>
       <c r="U20" s="6" t="n"/>
@@ -1832,13 +1988,21 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="n"/>
+      <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
+      <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="5" t="n"/>
       <c r="F21" s="5" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
@@ -1848,7 +2012,11 @@
       <c r="O21" s="6" t="n"/>
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="6" t="n"/>
-      <c r="R21" s="6" t="n"/>
+      <c r="R21" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S21" s="6" t="n"/>
       <c r="T21" s="6" t="n"/>
       <c r="U21" s="6" t="n"/>
@@ -1864,13 +2032,21 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="n"/>
+      <c r="B22" s="5" t="inlineStr"/>
       <c r="C22" s="5" t="n"/>
-      <c r="D22" s="5" t="n"/>
+      <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="5" t="n"/>
       <c r="F22" s="5" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H22" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I22" s="6" t="n"/>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
@@ -1880,7 +2056,11 @@
       <c r="O22" s="6" t="n"/>
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="6" t="n"/>
-      <c r="R22" s="6" t="n"/>
+      <c r="R22" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S22" s="6" t="n"/>
       <c r="T22" s="6" t="n"/>
       <c r="U22" s="6" t="n"/>
@@ -1896,13 +2076,21 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="n"/>
+      <c r="B23" s="5" t="inlineStr"/>
       <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
+      <c r="D23" s="5" t="inlineStr"/>
       <c r="E23" s="5" t="n"/>
       <c r="F23" s="5" t="n"/>
-      <c r="G23" s="6" t="n"/>
-      <c r="H23" s="6" t="n"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -1912,7 +2100,11 @@
       <c r="O23" s="6" t="n"/>
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="6" t="n"/>
-      <c r="R23" s="6" t="n"/>
+      <c r="R23" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S23" s="6" t="n"/>
       <c r="T23" s="6" t="n"/>
       <c r="U23" s="6" t="n"/>
@@ -1928,13 +2120,21 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="n"/>
+      <c r="B24" s="5" t="inlineStr"/>
       <c r="C24" s="5" t="n"/>
-      <c r="D24" s="5" t="n"/>
+      <c r="D24" s="5" t="inlineStr"/>
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="n"/>
-      <c r="G24" s="6" t="n"/>
-      <c r="H24" s="6" t="n"/>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H24" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I24" s="6" t="n"/>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
@@ -1944,7 +2144,11 @@
       <c r="O24" s="6" t="n"/>
       <c r="P24" s="6" t="n"/>
       <c r="Q24" s="6" t="n"/>
-      <c r="R24" s="6" t="n"/>
+      <c r="R24" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S24" s="6" t="n"/>
       <c r="T24" s="6" t="n"/>
       <c r="U24" s="6" t="n"/>
@@ -1960,13 +2164,21 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="n"/>
+      <c r="B25" s="5" t="inlineStr"/>
       <c r="C25" s="5" t="n"/>
-      <c r="D25" s="5" t="n"/>
+      <c r="D25" s="5" t="inlineStr"/>
       <c r="E25" s="5" t="n"/>
       <c r="F25" s="5" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
@@ -1976,7 +2188,11 @@
       <c r="O25" s="6" t="n"/>
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="6" t="n"/>
-      <c r="R25" s="6" t="n"/>
+      <c r="R25" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S25" s="6" t="n"/>
       <c r="T25" s="6" t="n"/>
       <c r="U25" s="6" t="n"/>
@@ -1992,13 +2208,21 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="n"/>
+      <c r="B26" s="5" t="inlineStr"/>
       <c r="C26" s="5" t="n"/>
-      <c r="D26" s="5" t="n"/>
+      <c r="D26" s="5" t="inlineStr"/>
       <c r="E26" s="5" t="n"/>
       <c r="F26" s="5" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H26" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I26" s="6" t="n"/>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
@@ -2008,7 +2232,11 @@
       <c r="O26" s="6" t="n"/>
       <c r="P26" s="6" t="n"/>
       <c r="Q26" s="6" t="n"/>
-      <c r="R26" s="6" t="n"/>
+      <c r="R26" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S26" s="6" t="n"/>
       <c r="T26" s="6" t="n"/>
       <c r="U26" s="6" t="n"/>
@@ -2024,13 +2252,21 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="n"/>
+      <c r="B27" s="5" t="inlineStr"/>
       <c r="C27" s="5" t="n"/>
-      <c r="D27" s="5" t="n"/>
+      <c r="D27" s="5" t="inlineStr"/>
       <c r="E27" s="5" t="n"/>
       <c r="F27" s="5" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
@@ -2040,7 +2276,11 @@
       <c r="O27" s="6" t="n"/>
       <c r="P27" s="6" t="n"/>
       <c r="Q27" s="6" t="n"/>
-      <c r="R27" s="6" t="n"/>
+      <c r="R27" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S27" s="6" t="n"/>
       <c r="T27" s="6" t="n"/>
       <c r="U27" s="6" t="n"/>
@@ -2056,13 +2296,21 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="n"/>
+      <c r="B28" s="5" t="inlineStr"/>
       <c r="C28" s="5" t="n"/>
-      <c r="D28" s="5" t="n"/>
+      <c r="D28" s="5" t="inlineStr"/>
       <c r="E28" s="5" t="n"/>
       <c r="F28" s="5" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I28" s="6" t="n"/>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
@@ -2072,7 +2320,11 @@
       <c r="O28" s="6" t="n"/>
       <c r="P28" s="6" t="n"/>
       <c r="Q28" s="6" t="n"/>
-      <c r="R28" s="6" t="n"/>
+      <c r="R28" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S28" s="6" t="n"/>
       <c r="T28" s="6" t="n"/>
       <c r="U28" s="6" t="n"/>
@@ -2088,13 +2340,21 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="n"/>
+      <c r="B29" s="5" t="inlineStr"/>
       <c r="C29" s="5" t="n"/>
-      <c r="D29" s="5" t="n"/>
+      <c r="D29" s="5" t="inlineStr"/>
       <c r="E29" s="5" t="n"/>
       <c r="F29" s="5" t="n"/>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H29" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
@@ -2104,7 +2364,11 @@
       <c r="O29" s="6" t="n"/>
       <c r="P29" s="6" t="n"/>
       <c r="Q29" s="6" t="n"/>
-      <c r="R29" s="6" t="n"/>
+      <c r="R29" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S29" s="6" t="n"/>
       <c r="T29" s="6" t="n"/>
       <c r="U29" s="6" t="n"/>
@@ -2120,13 +2384,21 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="n"/>
+      <c r="B30" s="5" t="inlineStr"/>
       <c r="C30" s="5" t="n"/>
-      <c r="D30" s="5" t="n"/>
+      <c r="D30" s="5" t="inlineStr"/>
       <c r="E30" s="5" t="n"/>
       <c r="F30" s="5" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H30" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I30" s="6" t="n"/>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
@@ -2136,7 +2408,11 @@
       <c r="O30" s="6" t="n"/>
       <c r="P30" s="6" t="n"/>
       <c r="Q30" s="6" t="n"/>
-      <c r="R30" s="6" t="n"/>
+      <c r="R30" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S30" s="6" t="n"/>
       <c r="T30" s="6" t="n"/>
       <c r="U30" s="6" t="n"/>
@@ -2152,13 +2428,21 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
-      <c r="B31" s="5" t="n"/>
+      <c r="B31" s="5" t="inlineStr"/>
       <c r="C31" s="5" t="n"/>
-      <c r="D31" s="5" t="n"/>
+      <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="5" t="n"/>
       <c r="F31" s="5" t="n"/>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
@@ -2168,7 +2452,11 @@
       <c r="O31" s="6" t="n"/>
       <c r="P31" s="6" t="n"/>
       <c r="Q31" s="6" t="n"/>
-      <c r="R31" s="6" t="n"/>
+      <c r="R31" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S31" s="6" t="n"/>
       <c r="T31" s="6" t="n"/>
       <c r="U31" s="6" t="n"/>
@@ -2184,13 +2472,21 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="n"/>
+      <c r="B32" s="5" t="inlineStr"/>
       <c r="C32" s="5" t="n"/>
-      <c r="D32" s="5" t="n"/>
+      <c r="D32" s="5" t="inlineStr"/>
       <c r="E32" s="5" t="n"/>
       <c r="F32" s="5" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>20260101</t>
+        </is>
+      </c>
+      <c r="H32" s="6" t="inlineStr">
+        <is>
+          <t>99991231</t>
+        </is>
+      </c>
       <c r="I32" s="6" t="n"/>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
@@ -2200,7 +2496,11 @@
       <c r="O32" s="6" t="n"/>
       <c r="P32" s="6" t="n"/>
       <c r="Q32" s="6" t="n"/>
-      <c r="R32" s="6" t="n"/>
+      <c r="R32" s="6" t="inlineStr">
+        <is>
+          <t>1,2,3,4,7</t>
+        </is>
+      </c>
       <c r="S32" s="6" t="n"/>
       <c r="T32" s="6" t="n"/>
       <c r="U32" s="6" t="n"/>

</xml_diff>

<commit_message>
Sync session21: extraction dedup fixes + generate_upload ITCD expansion
- rules/extraction_rules.py: Fix _find_sub_types_in_section newline normalization
  (PDF artifact "2종(계좌이체\n용)" → "2종(계좌이체용)", prevents duplicate sub_types)
- rules/extraction_rules.py: Fix _parse_age_table_separate_minmax dedup
  (3000-char window contained multiple sub_type tables, causing 2x-3x duplicate rows;
  2258 S00026: 36→16 rows)
- generate_upload.py: Expand rows per mapping entry (sub_type substring match + fallback)
  (2258 upload file: 1 ITCD pair → 13 pairs A01~A13 all present)
- generate_upload.py: Dedup by (UPPER, LOWER, data_tuple), completeness validation
- Regenerated all extracted/*.json, upload/*.xlsx, reports/*.xlsx, logs/*.json

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/upload/S00022_1228_연금저축_스마트하이드림연금보험.xlsx
+++ b/output/upload/S00022_1228_연금저축_스마트하이드림연금보험.xlsx
@@ -1436,41 +1436,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
@@ -1480,11 +1452,7 @@
       <c r="O8" s="6" t="n"/>
       <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R8" s="6" t="n"/>
       <c r="S8" s="6" t="n"/>
       <c r="T8" s="6" t="n"/>
       <c r="U8" s="6" t="n"/>
@@ -1500,41 +1468,13 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
       <c r="I9" s="6" t="n"/>
       <c r="J9" s="6" t="n"/>
       <c r="K9" s="6" t="n"/>
@@ -1544,11 +1484,7 @@
       <c r="O9" s="6" t="n"/>
       <c r="P9" s="6" t="n"/>
       <c r="Q9" s="6" t="n"/>
-      <c r="R9" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R9" s="6" t="n"/>
       <c r="S9" s="6" t="n"/>
       <c r="T9" s="6" t="n"/>
       <c r="U9" s="6" t="n"/>
@@ -1564,41 +1500,13 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
       <c r="I10" s="6" t="n"/>
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
@@ -1608,11 +1516,7 @@
       <c r="O10" s="6" t="n"/>
       <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R10" s="6" t="n"/>
       <c r="S10" s="6" t="n"/>
       <c r="T10" s="6" t="n"/>
       <c r="U10" s="6" t="n"/>
@@ -1628,41 +1532,13 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
       <c r="I11" s="6" t="n"/>
       <c r="J11" s="6" t="n"/>
       <c r="K11" s="6" t="n"/>
@@ -1672,11 +1548,7 @@
       <c r="O11" s="6" t="n"/>
       <c r="P11" s="6" t="n"/>
       <c r="Q11" s="6" t="n"/>
-      <c r="R11" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R11" s="6" t="n"/>
       <c r="S11" s="6" t="n"/>
       <c r="T11" s="6" t="n"/>
       <c r="U11" s="6" t="n"/>
@@ -1692,41 +1564,13 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G12" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
       <c r="I12" s="6" t="n"/>
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
@@ -1736,11 +1580,7 @@
       <c r="O12" s="6" t="n"/>
       <c r="P12" s="6" t="n"/>
       <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R12" s="6" t="n"/>
       <c r="S12" s="6" t="n"/>
       <c r="T12" s="6" t="n"/>
       <c r="U12" s="6" t="n"/>
@@ -1756,41 +1596,13 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n"/>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G13" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
       <c r="I13" s="6" t="n"/>
       <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="n"/>
@@ -1800,11 +1612,7 @@
       <c r="O13" s="6" t="n"/>
       <c r="P13" s="6" t="n"/>
       <c r="Q13" s="6" t="n"/>
-      <c r="R13" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R13" s="6" t="n"/>
       <c r="S13" s="6" t="n"/>
       <c r="T13" s="6" t="n"/>
       <c r="U13" s="6" t="n"/>
@@ -1820,41 +1628,13 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n"/>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
       <c r="I14" s="6" t="n"/>
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
@@ -1864,11 +1644,7 @@
       <c r="O14" s="6" t="n"/>
       <c r="P14" s="6" t="n"/>
       <c r="Q14" s="6" t="n"/>
-      <c r="R14" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R14" s="6" t="n"/>
       <c r="S14" s="6" t="n"/>
       <c r="T14" s="6" t="n"/>
       <c r="U14" s="6" t="n"/>
@@ -1884,41 +1660,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n"/>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
       <c r="I15" s="6" t="n"/>
       <c r="J15" s="6" t="n"/>
       <c r="K15" s="6" t="n"/>
@@ -1928,11 +1676,7 @@
       <c r="O15" s="6" t="n"/>
       <c r="P15" s="6" t="n"/>
       <c r="Q15" s="6" t="n"/>
-      <c r="R15" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R15" s="6" t="n"/>
       <c r="S15" s="6" t="n"/>
       <c r="T15" s="6" t="n"/>
       <c r="U15" s="6" t="n"/>
@@ -1948,41 +1692,13 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="n"/>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
       <c r="I16" s="6" t="n"/>
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
@@ -1992,11 +1708,7 @@
       <c r="O16" s="6" t="n"/>
       <c r="P16" s="6" t="n"/>
       <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R16" s="6" t="n"/>
       <c r="S16" s="6" t="n"/>
       <c r="T16" s="6" t="n"/>
       <c r="U16" s="6" t="n"/>
@@ -2012,41 +1724,13 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n"/>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
       <c r="I17" s="6" t="n"/>
       <c r="J17" s="6" t="n"/>
       <c r="K17" s="6" t="n"/>
@@ -2056,11 +1740,7 @@
       <c r="O17" s="6" t="n"/>
       <c r="P17" s="6" t="n"/>
       <c r="Q17" s="6" t="n"/>
-      <c r="R17" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R17" s="6" t="n"/>
       <c r="S17" s="6" t="n"/>
       <c r="T17" s="6" t="n"/>
       <c r="U17" s="6" t="n"/>
@@ -2076,41 +1756,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
       <c r="I18" s="6" t="n"/>
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
@@ -2120,11 +1772,7 @@
       <c r="O18" s="6" t="n"/>
       <c r="P18" s="6" t="n"/>
       <c r="Q18" s="6" t="n"/>
-      <c r="R18" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R18" s="6" t="n"/>
       <c r="S18" s="6" t="n"/>
       <c r="T18" s="6" t="n"/>
       <c r="U18" s="6" t="n"/>
@@ -2140,41 +1788,13 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n"/>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F19" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
       <c r="I19" s="6" t="n"/>
       <c r="J19" s="6" t="n"/>
       <c r="K19" s="6" t="n"/>
@@ -2184,11 +1804,7 @@
       <c r="O19" s="6" t="n"/>
       <c r="P19" s="6" t="n"/>
       <c r="Q19" s="6" t="n"/>
-      <c r="R19" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R19" s="6" t="n"/>
       <c r="S19" s="6" t="n"/>
       <c r="T19" s="6" t="n"/>
       <c r="U19" s="6" t="n"/>
@@ -2204,41 +1820,13 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="n"/>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
       <c r="I20" s="6" t="n"/>
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
@@ -2248,11 +1836,7 @@
       <c r="O20" s="6" t="n"/>
       <c r="P20" s="6" t="n"/>
       <c r="Q20" s="6" t="n"/>
-      <c r="R20" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R20" s="6" t="n"/>
       <c r="S20" s="6" t="n"/>
       <c r="T20" s="6" t="n"/>
       <c r="U20" s="6" t="n"/>
@@ -2268,41 +1852,13 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n"/>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F21" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
       <c r="I21" s="6" t="n"/>
       <c r="J21" s="6" t="n"/>
       <c r="K21" s="6" t="n"/>
@@ -2312,11 +1868,7 @@
       <c r="O21" s="6" t="n"/>
       <c r="P21" s="6" t="n"/>
       <c r="Q21" s="6" t="n"/>
-      <c r="R21" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R21" s="6" t="n"/>
       <c r="S21" s="6" t="n"/>
       <c r="T21" s="6" t="n"/>
       <c r="U21" s="6" t="n"/>
@@ -2332,41 +1884,13 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n"/>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
       <c r="I22" s="6" t="n"/>
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
@@ -2376,11 +1900,7 @@
       <c r="O22" s="6" t="n"/>
       <c r="P22" s="6" t="n"/>
       <c r="Q22" s="6" t="n"/>
-      <c r="R22" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R22" s="6" t="n"/>
       <c r="S22" s="6" t="n"/>
       <c r="T22" s="6" t="n"/>
       <c r="U22" s="6" t="n"/>
@@ -2396,41 +1916,13 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n"/>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F23" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
       <c r="I23" s="6" t="n"/>
       <c r="J23" s="6" t="n"/>
       <c r="K23" s="6" t="n"/>
@@ -2440,11 +1932,7 @@
       <c r="O23" s="6" t="n"/>
       <c r="P23" s="6" t="n"/>
       <c r="Q23" s="6" t="n"/>
-      <c r="R23" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R23" s="6" t="n"/>
       <c r="S23" s="6" t="n"/>
       <c r="T23" s="6" t="n"/>
       <c r="U23" s="6" t="n"/>
@@ -2460,41 +1948,13 @@
     </row>
     <row r="24">
       <c r="A24" s="5" t="n"/>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
       <c r="I24" s="6" t="n"/>
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
@@ -2504,11 +1964,7 @@
       <c r="O24" s="6" t="n"/>
       <c r="P24" s="6" t="n"/>
       <c r="Q24" s="6" t="n"/>
-      <c r="R24" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R24" s="6" t="n"/>
       <c r="S24" s="6" t="n"/>
       <c r="T24" s="6" t="n"/>
       <c r="U24" s="6" t="n"/>
@@ -2524,41 +1980,13 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="n"/>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
       <c r="I25" s="6" t="n"/>
       <c r="J25" s="6" t="n"/>
       <c r="K25" s="6" t="n"/>
@@ -2568,11 +1996,7 @@
       <c r="O25" s="6" t="n"/>
       <c r="P25" s="6" t="n"/>
       <c r="Q25" s="6" t="n"/>
-      <c r="R25" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R25" s="6" t="n"/>
       <c r="S25" s="6" t="n"/>
       <c r="T25" s="6" t="n"/>
       <c r="U25" s="6" t="n"/>
@@ -2588,41 +2012,13 @@
     </row>
     <row r="26">
       <c r="A26" s="5" t="n"/>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H26" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
       <c r="I26" s="6" t="n"/>
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
@@ -2632,11 +2028,7 @@
       <c r="O26" s="6" t="n"/>
       <c r="P26" s="6" t="n"/>
       <c r="Q26" s="6" t="n"/>
-      <c r="R26" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R26" s="6" t="n"/>
       <c r="S26" s="6" t="n"/>
       <c r="T26" s="6" t="n"/>
       <c r="U26" s="6" t="n"/>
@@ -2652,41 +2044,13 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n"/>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G27" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
       <c r="I27" s="6" t="n"/>
       <c r="J27" s="6" t="n"/>
       <c r="K27" s="6" t="n"/>
@@ -2696,11 +2060,7 @@
       <c r="O27" s="6" t="n"/>
       <c r="P27" s="6" t="n"/>
       <c r="Q27" s="6" t="n"/>
-      <c r="R27" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R27" s="6" t="n"/>
       <c r="S27" s="6" t="n"/>
       <c r="T27" s="6" t="n"/>
       <c r="U27" s="6" t="n"/>
@@ -2716,41 +2076,13 @@
     </row>
     <row r="28">
       <c r="A28" s="5" t="n"/>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E28" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H28" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
       <c r="I28" s="6" t="n"/>
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
@@ -2760,11 +2092,7 @@
       <c r="O28" s="6" t="n"/>
       <c r="P28" s="6" t="n"/>
       <c r="Q28" s="6" t="n"/>
-      <c r="R28" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R28" s="6" t="n"/>
       <c r="S28" s="6" t="n"/>
       <c r="T28" s="6" t="n"/>
       <c r="U28" s="6" t="n"/>
@@ -2780,41 +2108,13 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="n"/>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F29" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
       <c r="I29" s="6" t="n"/>
       <c r="J29" s="6" t="n"/>
       <c r="K29" s="6" t="n"/>
@@ -2824,11 +2124,7 @@
       <c r="O29" s="6" t="n"/>
       <c r="P29" s="6" t="n"/>
       <c r="Q29" s="6" t="n"/>
-      <c r="R29" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R29" s="6" t="n"/>
       <c r="S29" s="6" t="n"/>
       <c r="T29" s="6" t="n"/>
       <c r="U29" s="6" t="n"/>
@@ -2844,41 +2140,13 @@
     </row>
     <row r="30">
       <c r="A30" s="5" t="n"/>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G30" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H30" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
       <c r="I30" s="6" t="n"/>
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
@@ -2888,11 +2156,7 @@
       <c r="O30" s="6" t="n"/>
       <c r="P30" s="6" t="n"/>
       <c r="Q30" s="6" t="n"/>
-      <c r="R30" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R30" s="6" t="n"/>
       <c r="S30" s="6" t="n"/>
       <c r="T30" s="6" t="n"/>
       <c r="U30" s="6" t="n"/>
@@ -2908,41 +2172,13 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="n"/>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G31" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
       <c r="I31" s="6" t="n"/>
       <c r="J31" s="6" t="n"/>
       <c r="K31" s="6" t="n"/>
@@ -2952,11 +2188,7 @@
       <c r="O31" s="6" t="n"/>
       <c r="P31" s="6" t="n"/>
       <c r="Q31" s="6" t="n"/>
-      <c r="R31" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R31" s="6" t="n"/>
       <c r="S31" s="6" t="n"/>
       <c r="T31" s="6" t="n"/>
       <c r="U31" s="6" t="n"/>
@@ -2972,41 +2204,13 @@
     </row>
     <row r="32">
       <c r="A32" s="5" t="n"/>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>1228137</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>한화생명 연금저축 스마트하이드림연금보험 종신연금형</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>S00022</t>
-        </is>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>20260101</t>
-        </is>
-      </c>
-      <c r="H32" s="6" t="inlineStr">
-        <is>
-          <t>99991231</t>
-        </is>
-      </c>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="6" t="n"/>
       <c r="I32" s="6" t="n"/>
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
@@ -3016,11 +2220,7 @@
       <c r="O32" s="6" t="n"/>
       <c r="P32" s="6" t="n"/>
       <c r="Q32" s="6" t="n"/>
-      <c r="R32" s="6" t="inlineStr">
-        <is>
-          <t>1,2,3,4,7</t>
-        </is>
-      </c>
+      <c r="R32" s="6" t="n"/>
       <c r="S32" s="6" t="n"/>
       <c r="T32" s="6" t="n"/>
       <c r="U32" s="6" t="n"/>

</xml_diff>